<commit_message>
Price natural flavors at $70/gal per client direction
Updates the generic natural-flavor cost basis from a researched ~$40/kg
estimate to a client-directed $70/gal (normalized to $8.39/lb at SG 1.0).
Recomputes per-can and per-case ingredient costs across all four formulas.

https://claude.ai/code/session_01Xys6L7LsgSa2ACDzAaru9U
</commit_message>
<xml_diff>
--- a/STH_Run001_Ingredient_Cost_Per_Can.xlsx
+++ b/STH_Run001_Ingredient_Cost_Per_Can.xlsx
@@ -667,7 +667,7 @@
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>the Gold Coast flavors, chamomile hydrosol, lemon verbena). These are the biggest swing factors — replace with actual</t>
+          <t>chamomile hydrosol, lemon verbena). Natural flavors are set per client direction at $70/gal (SG 1.0 assumed). These are</t>
         </is>
       </c>
     </row>
@@ -1082,29 +1082,29 @@
       <c r="B14" s="9" t="n">
         <v>0.399</v>
       </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>18.14</v>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.016</v>
+        <v>0.0074</v>
       </c>
       <c r="G14" s="11">
         <f>F14/$F$19</f>
         <v/>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -1117,29 +1117,29 @@
       <c r="B15" s="9" t="n">
         <v>0.578</v>
       </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>18.14</v>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F15" s="10" t="n">
-        <v>0.0231</v>
+        <v>0.0107</v>
       </c>
       <c r="G15" s="11">
         <f>F15/$F$19</f>
         <v/>
       </c>
-      <c r="H15" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -1152,29 +1152,29 @@
       <c r="B16" s="9" t="n">
         <v>0.158</v>
       </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>18.14</v>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F16" s="10" t="n">
-        <v>0.0063</v>
+        <v>0.0029</v>
       </c>
       <c r="G16" s="11">
         <f>F16/$F$19</f>
         <v/>
       </c>
-      <c r="H16" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -1187,29 +1187,29 @@
       <c r="B17" s="9" t="n">
         <v>0.504</v>
       </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="n">
-        <v>18.14</v>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F17" s="10" t="n">
-        <v>0.0202</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="G17" s="11">
         <f>F17/$F$19</f>
         <v/>
       </c>
-      <c r="H17" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -1290,10 +1290,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1698,29 +1694,29 @@
       <c r="B14" s="9" t="n">
         <v>0.399</v>
       </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>18.14</v>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.016</v>
+        <v>0.0074</v>
       </c>
       <c r="G14" s="11">
         <f>F14/$F$19</f>
         <v/>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -1733,29 +1729,29 @@
       <c r="B15" s="9" t="n">
         <v>0.242</v>
       </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>18.14</v>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F15" s="10" t="n">
-        <v>0.0097</v>
+        <v>0.0045</v>
       </c>
       <c r="G15" s="11">
         <f>F15/$F$19</f>
         <v/>
       </c>
-      <c r="H15" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -1768,29 +1764,29 @@
       <c r="B16" s="9" t="n">
         <v>0.714</v>
       </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>18.14</v>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F16" s="10" t="n">
-        <v>0.0286</v>
+        <v>0.0132</v>
       </c>
       <c r="G16" s="11">
         <f>F16/$F$19</f>
         <v/>
       </c>
-      <c r="H16" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -1803,29 +1799,29 @@
       <c r="B17" s="9" t="n">
         <v>0.368</v>
       </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="n">
-        <v>18.14</v>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F17" s="10" t="n">
-        <v>0.0147</v>
+        <v>0.0068</v>
       </c>
       <c r="G17" s="11">
         <f>F17/$F$19</f>
         <v/>
       </c>
-      <c r="H17" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -1906,10 +1902,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId4"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2279,29 +2271,29 @@
       <c r="B13" s="9" t="n">
         <v>1.193</v>
       </c>
-      <c r="C13" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="n">
-        <v>18.14</v>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F13" s="10" t="n">
-        <v>0.0477</v>
+        <v>0.0221</v>
       </c>
       <c r="G13" s="11">
         <f>F13/$F$19</f>
         <v/>
       </c>
-      <c r="H13" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H13" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -2314,29 +2306,29 @@
       <c r="B14" s="9" t="n">
         <v>0.895</v>
       </c>
-      <c r="C14" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="n">
-        <v>18.14</v>
+      <c r="C14" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D14" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E14" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F14" s="10" t="n">
-        <v>0.0358</v>
+        <v>0.0165</v>
       </c>
       <c r="G14" s="11">
         <f>F14/$F$19</f>
         <v/>
       </c>
-      <c r="H14" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H14" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -2349,29 +2341,29 @@
       <c r="B15" s="9" t="n">
         <v>0.142</v>
       </c>
-      <c r="C15" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D15" s="13" t="n">
-        <v>18.14</v>
+      <c r="C15" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D15" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E15" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F15" s="10" t="n">
-        <v>0.0057</v>
+        <v>0.0026</v>
       </c>
       <c r="G15" s="11">
         <f>F15/$F$19</f>
         <v/>
       </c>
-      <c r="H15" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H15" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -2384,29 +2376,29 @@
       <c r="B16" s="9" t="n">
         <v>0.358</v>
       </c>
-      <c r="C16" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D16" s="13" t="n">
-        <v>18.14</v>
+      <c r="C16" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D16" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E16" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F16" s="10" t="n">
-        <v>0.0143</v>
+        <v>0.0066</v>
       </c>
       <c r="G16" s="11">
         <f>F16/$F$19</f>
         <v/>
       </c>
-      <c r="H16" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H16" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -2419,29 +2411,29 @@
       <c r="B17" s="9" t="n">
         <v>0.716</v>
       </c>
-      <c r="C17" s="13" t="inlineStr">
-        <is>
-          <t>$40.00 /kg</t>
-        </is>
-      </c>
-      <c r="D17" s="13" t="n">
-        <v>18.14</v>
+      <c r="C17" s="9" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D17" s="9" t="n">
+        <v>8.390000000000001</v>
       </c>
       <c r="E17" s="9" t="inlineStr">
         <is>
-          <t>~4 lb</t>
+          <t>1 gal</t>
         </is>
       </c>
       <c r="F17" s="10" t="n">
-        <v>0.0286</v>
+        <v>0.0132</v>
       </c>
       <c r="G17" s="11">
         <f>F17/$F$19</f>
         <v/>
       </c>
-      <c r="H17" s="14" t="inlineStr">
-        <is>
-          <t>Katana flavor avg + FlavorConcentrates bulk</t>
+      <c r="H17" s="12" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
       </c>
     </row>
@@ -2521,11 +2513,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H13" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H14" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H15" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H16" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H17" r:id="rId9"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Rebuild costing from Spec tabs (recipes were wrong)
The Quoting tabs are unreliable: Serenity dropped an ingredient and
mis-aligned quantities, The Fountain used the wrong can size and a scrambled
list, and Defend carried a completely different placeholder recipe. Recipes
are now taken from the four Spec tabs (embedded-image formulas). All products
are 250 mL / 12-pack. Spec grams are exact; a separate +5% line covers yield
loss. Adds vegetable glycerin pricing for Defend.

https://claude.ai/code/session_01Xys6L7LsgSa2ACDzAaru9U
</commit_message>
<xml_diff>
--- a/STH_Run001_Ingredient_Cost_Per_Can.xlsx
+++ b/STH_Run001_Ingredient_Cost_Per_Can.xlsx
@@ -20,12 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="$0.0000"/>
-    <numFmt numFmtId="165" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="$0.00"/>
+  <numFmts count="4">
+    <numFmt numFmtId="164" formatCode="0.000"/>
+    <numFmt numFmtId="165" formatCode="$0.0000"/>
+    <numFmt numFmtId="166" formatCode="0.0%"/>
+    <numFmt numFmtId="167" formatCode="$0.00"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -58,6 +59,9 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <i val="1"/>
     </font>
   </fonts>
   <fills count="4">
@@ -104,7 +108,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment wrapText="1"/>
@@ -124,13 +128,16 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -144,9 +151,11 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="6" fillId="3" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -513,16 +522,16 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A25"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="120" customWidth="1" min="1" max="1"/>
+    <col width="122" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Southern Tier Hemp — Run 001  |  Ingredient cost per can</t>
+          <t>Southern Tier Hemp — Run 001  |  Ingredient cost per can (rebuilt from Spec tabs)</t>
         </is>
       </c>
     </row>
@@ -539,21 +548,21 @@
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
         <is>
-          <t>What this is</t>
+          <t>Source of recipes</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>One tab per formula (Showtime Elixir, Serenity, The Fountain, Defend). Each lists every ingredient with its native unit price,</t>
+          <t>Recipes are taken from the four "Spec - &lt;product&gt;" tabs, whose formulas are stored as embedded IMAGES (not cell values).</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>a normalized cost/lb, MOQ, the cost contributed per can, and a source. Totals give ingredient cost per can and per case.</t>
+          <t>All four products are 250 mL fill, 12 cans/pack, 100% case yield = 15,141.6 cans per 3,785.41 L (1,000 gal) batch.</t>
         </is>
       </c>
     </row>
@@ -563,118 +572,104 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Why prices were rebuilt (important)</t>
+          <t>Why the earlier version was wrong</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>1) On the original Quoting tabs the Cost/Unit column is placeholder data: the same four values ($5.56/$2.91/$0.58/$2.91, MOQ</t>
+          <t>The first workbook was built from the "Quoting - &lt;product&gt;" tabs, which are unreliable: (1) Serenity dropped "Organic</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   275/51/2500/51) repeat identically down all four products regardless of ingredient (e.g. "Potassium Benzoate" carried</t>
+          <t>Chamomile Flavor" and mis-aligned the bottom quantities; (2) The Fountain was set to 355 mL with a scrambled list;</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">   GNS-95% pricing). Only Water ($0.10/gal) was a real number.</t>
+          <t>(3) Defend carried a completely different placeholder recipe (GNS/sugar/verbena at 1,000 gal); (4) the Cost/Unit column</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>2) The Cases input was blank, so every per-can / MOQ formula returned #DIV/0! — the tabs could not output a cost.</t>
+          <t>repeated the same four placeholder prices down every product. This version ignores the Quoting tabs for recipe + price.</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="3" t="inlineStr">
-        <is>
-          <t>Prices here were sourced first from your internal data (Katana avg cost; the "Complete Ingredients w Pricing" tab), then from</t>
-        </is>
-      </c>
+      <c r="A13" s="3" t="inlineStr"/>
     </row>
     <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>web research for the proprietary items those sheets do not price. Source of each price is in the Source column (links where external).</t>
+      <c r="A14" s="4" t="inlineStr">
+        <is>
+          <t>Method</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="3" t="inlineStr"/>
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Cost/can = (spec g/can / 453.592) x cost/lb.  Cost/lb normalization: $/kg x 0.4536; $/gal / (8.345 x SG); $/lb as-is.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
-      <c r="A16" s="4" t="inlineStr">
-        <is>
-          <t>Method</t>
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Spec g/can shown are exact (match the spec). A separate line adds 5% for production/yield loss (what you must purchase).</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>Cost/can = (spec amount, lb) x per-can multiplier x cost/lb.  Per-can multiplier k = (can_L x 1.05 loss) / (spec-batch_L).</t>
+          <t>Natural flavors (Gold Coast / FONA) priced per client direction at $70/gal (SG 1.0). Signature Beverage Enhancer kept at</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>Cost/lb normalization: $/kg x 0.4536; $/gal / (8.345 x specific gravity); $/lb used as-is.</t>
+          <t>a separate $34/lb estimate (say the word to move it to $70/gal too).</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>This is the linear (marginal) ingredient cost — what the liquid costs per can at scale. It does NOT load minimum-order</t>
-        </is>
-      </c>
+      <c r="A19" s="3" t="inlineStr"/>
     </row>
     <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>quantities; for a single small run, buying full MOQs (e.g. 275 lb preservative, 25 kg color) would raise the effective per-can cost.</t>
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>Confidence</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="3" t="inlineStr"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Orange cells = researched estimates (CBD Hydrobond, Talin PG95, natural colors, chamomile hydrosol, vegetable glycerin,</t>
+        </is>
+      </c>
     </row>
     <row r="22">
-      <c r="A22" s="4" t="inlineStr">
-        <is>
-          <t>Confidence</t>
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Signature Enhancer). Biggest swing factors: Serenity chamomile hydrosol (~$0.22/can) and Talin. Firm: water, citric acid,</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>Orange cells = researched estimates with no firm internal/quoted price (CBD Hydrobond, Talin PG95, the natural colors,</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>chamomile hydrosol, lemon verbena). Natural flavors are set per client direction at $70/gal (SG 1.0 assumed). These are</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="3" t="inlineStr">
-        <is>
-          <t>purchase costs to finalize. Commodity/internal items (water, citric acid, sugar, GNS, juice, preservatives) are firm.</t>
+          <t>fructose, preservatives, Bossen lychee. Replace orange items with actual purchase costs to finalize.</t>
         </is>
       </c>
     </row>
@@ -689,17 +684,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -712,19 +707,19 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>250 mL can | 24/case | 5% production-loss adj included | linear (marginal) ingredient cost, MOQ not loaded</t>
+          <t>250 mL fill | 12-pack | source: Spec tab (embedded image). Spec g/can are exact; cost = spec x cost/lb (no loss). Loss line below.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Ingredient</t>
+          <t>Ingredient (per spec)</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Amt/can (g)</t>
+          <t>Spec g/can</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -734,7 +729,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Cost/lb ($)</t>
+          <t>Cost/lb $</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -744,12 +739,12 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Cost/can ($)</t>
+          <t>Cost/can $</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>% of ing. cost</t>
+          <t>% ing.</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -761,35 +756,35 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Treated Water (RO)</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>257.278</v>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
+        <v>245</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>$0.10 /gal</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="10" t="n">
         <v>0.01</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F5" s="10" t="n">
-        <v>0.0068</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="F5" s="11" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="G5" s="12">
         <f>F5/$F$19</f>
         <v/>
       </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>Internal: spec sheet (Drayhorse)</t>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Internal: spec sheet (Drayhorse RO)</t>
         </is>
       </c>
     </row>
@@ -800,29 +795,29 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
+        <v>0.075</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>$4.82 /kg</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="10" t="n">
         <v>2.19</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>~55 lb</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n">
+      <c r="F6" s="11" t="n">
         <v>0.0004</v>
       </c>
-      <c r="G6" s="11">
+      <c r="G6" s="12">
         <f>F6/$F$19</f>
         <v/>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>Internal: Katana avg cost</t>
         </is>
@@ -835,29 +830,29 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
+        <v>0.075</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>$2.86 /kg</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10" t="n">
         <v>1.3</v>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>55 lb</t>
         </is>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <v>0.0002</v>
       </c>
-      <c r="G7" s="11">
+      <c r="G7" s="12">
         <f>F7/$F$19</f>
         <v/>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>Internal: Katana avg cost</t>
         </is>
@@ -866,35 +861,35 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Grape Blue Shade 183922</t>
+          <t>GNT USA Grape Blue Shade 183922</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>0.132</v>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
+        <v>0.126</v>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>$55.00 /kg</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>24.95</v>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>~25 kg</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n">
-        <v>0.0073</v>
-      </c>
-      <c r="G8" s="11">
+      <c r="F8" s="11" t="n">
+        <v>0.0069</v>
+      </c>
+      <c r="G8" s="12">
         <f>F8/$F$19</f>
         <v/>
       </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>GNT EXBERRY (natural color, est.)</t>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>GNT EXBERRY natural color (est.)</t>
         </is>
       </c>
     </row>
@@ -905,101 +900,101 @@
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.052</v>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
+        <v>0.05</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>$300.00 /kg</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>136.08</v>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>1 kg</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n">
-        <v>0.0157</v>
-      </c>
-      <c r="G9" s="11">
+      <c r="F9" s="11" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G9" s="12">
         <f>F9/$F$19</f>
         <v/>
       </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>Hemp Depot (water-soluble CBD powder)</t>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>Hemp Depot water-soluble CBD (est.)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Bossen Lychee Concentrated Syrup</t>
+          <t>Bossen Lychee Conc. Syrup 535SYPLYCH-SM</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>1.313</v>
-      </c>
-      <c r="C10" s="9" t="inlineStr">
+        <v>1.25</v>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
         <is>
           <t>$15.45 /lb</t>
         </is>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="10" t="n">
         <v>15.45</v>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>5.5 lb</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n">
-        <v>0.0447</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="F10" s="11" t="n">
+        <v>0.0426</v>
+      </c>
+      <c r="G10" s="12">
         <f>F10/$F$19</f>
         <v/>
       </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>Boba Warehouse / Amazon ($85 / 5.5 lb)</t>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Boba Warehouse ($85 / 5.5 lb)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Talin PG95 T0001</t>
+          <t>Talin PG95 T0001 (Naturex)</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>0.368</v>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
+        <v>0.35</v>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>$200.00 /kg</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>90.72</v>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>1 kg</t>
         </is>
       </c>
-      <c r="F11" s="10" t="n">
-        <v>0.0735</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="F11" s="11" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G11" s="12">
         <f>F11/$F$19</f>
         <v/>
       </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>Knowde (Naturex/Givaudan Talin) + bulk thaumatin</t>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Naturex/Givaudan Talin; bulk thaumatin (est.)</t>
         </is>
       </c>
     </row>
@@ -1010,29 +1005,29 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>$1.20 /lb</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <v>1.2</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>50 lb</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="G12" s="11">
+      <c r="F12" s="11" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="G12" s="12">
         <f>F12/$F$19</f>
         <v/>
       </c>
-      <c r="H12" s="14" t="inlineStr">
+      <c r="H12" s="15" t="inlineStr">
         <is>
           <t>Bakers Authority (ADM Cornsweet)</t>
         </is>
@@ -1045,29 +1040,29 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.242</v>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
+        <v>0.23</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>$1.52 /lb</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="10" t="n">
         <v>1.52</v>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>50 lb</t>
         </is>
       </c>
-      <c r="F13" s="10" t="n">
+      <c r="F13" s="11" t="n">
         <v>0.0008</v>
       </c>
-      <c r="G13" s="11">
+      <c r="G13" s="12">
         <f>F13/$F$19</f>
         <v/>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Internal: Complete Ingredients tab (Brenntag)</t>
         </is>
@@ -1076,33 +1071,33 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Ultra Masking Natural Flavor</t>
+          <t>Ultra Masking Nat 380223 (Gold Coast)</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.399</v>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
+        <v>0.38</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
-        <v>0.0074</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="F14" s="11" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="G14" s="12">
         <f>F14/$F$19</f>
         <v/>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -1111,33 +1106,33 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Natural Lychee Flavor</t>
+          <t>Natural Lychee 348692 (Gold Coast)</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.578</v>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
+        <v>0.55</v>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F15" s="10" t="n">
-        <v>0.0107</v>
-      </c>
-      <c r="G15" s="11">
+      <c r="F15" s="11" t="n">
+        <v>0.0102</v>
+      </c>
+      <c r="G15" s="12">
         <f>F15/$F$19</f>
         <v/>
       </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -1146,33 +1141,33 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Organic Lemon (flavor)</t>
+          <t>Organic Lemon 601032 (Gold Coast)</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>0.158</v>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
+        <v>0.15</v>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n">
-        <v>0.0029</v>
-      </c>
-      <c r="G16" s="11">
+      <c r="F16" s="11" t="n">
+        <v>0.0028</v>
+      </c>
+      <c r="G16" s="12">
         <f>F16/$F$19</f>
         <v/>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -1181,33 +1176,33 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Pink Grapefruit (flavor)</t>
+          <t>Pink Grapefruit 606817 (Gold Coast)</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>0.504</v>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
+        <v>0.48</v>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F17" s="10" t="n">
-        <v>0.009299999999999999</v>
-      </c>
-      <c r="G17" s="11">
+      <c r="F17" s="11" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="G17" s="12">
         <f>F17/$F$19</f>
         <v/>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -1216,70 +1211,81 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Signature Beverage Enhancer</t>
+          <t>Signature Beverage Enhancer (Blue Pacific)</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>0.08400000000000001</v>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
+        <v>0.08</v>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>$34.00 /lb</t>
         </is>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>1 lb</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n">
-        <v>0.0063</v>
-      </c>
-      <c r="G18" s="11">
+      <c r="F18" s="11" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="G18" s="12">
         <f>F18/$F$19</f>
         <v/>
       </c>
-      <c r="H18" s="12" t="inlineStr">
-        <is>
-          <t>Internal: Complete Ingredients tab (Signature Flavors analog)</t>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Blue Pacific Flavors analog (est.)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>TOTAL ingredient cost / can</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n"/>
-      <c r="C19" s="16" t="n"/>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="17">
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="17" t="n"/>
+      <c r="F19" s="18">
         <f>SUM(F5:F18)</f>
         <v/>
       </c>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
+      <c r="G19" s="17" t="n"/>
+      <c r="H19" s="17" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Cost / 24-can case</t>
-        </is>
-      </c>
-      <c r="F20" s="19">
-        <f>F19*24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>Orange = researched estimate (no firm internal/quoted price). Tighten with actual PO/invoice cost.</t>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + 5% production-loss (purchasing basis)</t>
+        </is>
+      </c>
+      <c r="F20" s="20">
+        <f>F19*1.05</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Cost / 12-pack (with loss)</t>
+        </is>
+      </c>
+      <c r="F21" s="22">
+        <f>F20*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>Orange = researched estimate (no firm internal/quoted price). Replace with actual PO cost to finalize.</t>
         </is>
       </c>
     </row>
@@ -1301,17 +1307,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1324,19 +1330,19 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>250 mL can | 24/case | 5% production-loss adj included | linear (marginal) ingredient cost, MOQ not loaded</t>
+          <t>250 mL fill | 12-pack | source: Spec tab (embedded image). Spec g/can are exact; cost = spec x cost/lb (no loss). Loss line below.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Ingredient</t>
+          <t>Ingredient (per spec)</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Amt/can (g)</t>
+          <t>Spec g/can</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -1346,7 +1352,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Cost/lb ($)</t>
+          <t>Cost/lb $</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1356,12 +1362,12 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Cost/can ($)</t>
+          <t>Cost/can $</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>% of ing. cost</t>
+          <t>% ing.</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -1373,68 +1379,68 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Treated Water (RO)</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>238.586</v>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
+        <v>227.2</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>$0.10 /gal</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="10" t="n">
         <v>0.01</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F5" s="10" t="n">
-        <v>0.0063</v>
-      </c>
-      <c r="G5" s="11">
-        <f>F5/$F$19</f>
-        <v/>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>Internal: spec sheet (Drayhorse)</t>
+      <c r="F5" s="11" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="G5" s="12">
+        <f>F5/$F$20</f>
+        <v/>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Internal: spec sheet (Drayhorse RO)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>Chamomile Hydrosol</t>
+          <t>Chamomile Hydrosol (DOFON)</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>17.642</v>
-      </c>
-      <c r="C6" s="13" t="inlineStr">
+        <v>16.8</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
         <is>
           <t>$50.00 /gal</t>
         </is>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="14" t="n">
         <v>5.99</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n">
-        <v>0.233</v>
-      </c>
-      <c r="G6" s="11">
-        <f>F6/$F$19</f>
-        <v/>
-      </c>
-      <c r="H6" s="14" t="inlineStr">
+      <c r="F6" s="11" t="n">
+        <v>0.2219</v>
+      </c>
+      <c r="G6" s="12">
+        <f>F6/$F$20</f>
+        <v/>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
         <is>
           <t>Mountain Rose Herbs (est.)</t>
         </is>
@@ -1447,29 +1453,29 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
+        <v>0.075</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>$4.82 /kg</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10" t="n">
         <v>2.19</v>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>~55 lb</t>
         </is>
       </c>
-      <c r="F7" s="10" t="n">
+      <c r="F7" s="11" t="n">
         <v>0.0004</v>
       </c>
-      <c r="G7" s="11">
-        <f>F7/$F$19</f>
-        <v/>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="G7" s="12">
+        <f>F7/$F$20</f>
+        <v/>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>Internal: Katana avg cost</t>
         </is>
@@ -1482,29 +1488,29 @@
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>0.079</v>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
+        <v>0.075</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
         <is>
           <t>$2.86 /kg</t>
         </is>
       </c>
-      <c r="D8" s="9" t="n">
+      <c r="D8" s="10" t="n">
         <v>1.3</v>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>55 lb</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n">
+      <c r="F8" s="11" t="n">
         <v>0.0002</v>
       </c>
-      <c r="G8" s="11">
-        <f>F8/$F$19</f>
-        <v/>
-      </c>
-      <c r="H8" s="12" t="inlineStr">
+      <c r="G8" s="12">
+        <f>F8/$F$20</f>
+        <v/>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
         <is>
           <t>Internal: Katana avg cost</t>
         </is>
@@ -1513,105 +1519,105 @@
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Grape Blue Shade</t>
+          <t>GNT USA Grape Blue Shade 183922</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.237</v>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
+        <v>0.226</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>$55.00 /kg</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>24.95</v>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>~25 kg</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n">
-        <v>0.0131</v>
-      </c>
-      <c r="G9" s="11">
-        <f>F9/$F$19</f>
-        <v/>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>GNT EXBERRY (natural color, est.)</t>
+      <c r="F9" s="11" t="n">
+        <v>0.0124</v>
+      </c>
+      <c r="G9" s="12">
+        <f>F9/$F$20</f>
+        <v/>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>GNT EXBERRY natural color (est.)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>CBD Hydrobond</t>
+          <t>CBD Hydrobond 685449</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.053</v>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
+        <v>0.05</v>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>$300.00 /kg</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>136.08</v>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>1 kg</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n">
-        <v>0.0158</v>
-      </c>
-      <c r="G10" s="11">
-        <f>F10/$F$19</f>
-        <v/>
-      </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>Hemp Depot (water-soluble CBD powder)</t>
+      <c r="F10" s="11" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G10" s="12">
+        <f>F10/$F$20</f>
+        <v/>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Hemp Depot water-soluble CBD (est.)</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="8" t="inlineStr">
         <is>
-          <t>Talin PG95</t>
+          <t>Talin PG95 T0001 (Naturex)</t>
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>0.473</v>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
+        <v>0.45</v>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>$200.00 /kg</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>90.72</v>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>1 kg</t>
         </is>
       </c>
-      <c r="F11" s="10" t="n">
-        <v>0.0945</v>
-      </c>
-      <c r="G11" s="11">
-        <f>F11/$F$19</f>
-        <v/>
-      </c>
-      <c r="H11" s="14" t="inlineStr">
-        <is>
-          <t>Knowde (Naturex/Givaudan Talin) + bulk thaumatin</t>
+      <c r="F11" s="11" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G11" s="12">
+        <f>F11/$F$20</f>
+        <v/>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Naturex/Givaudan Talin; bulk thaumatin (est.)</t>
         </is>
       </c>
     </row>
@@ -1622,29 +1628,29 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="C12" s="13" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
         <is>
           <t>$1.20 /lb</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="14" t="n">
         <v>1.2</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>50 lb</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
-        <v>0.0028</v>
-      </c>
-      <c r="G12" s="11">
-        <f>F12/$F$19</f>
-        <v/>
-      </c>
-      <c r="H12" s="14" t="inlineStr">
+      <c r="F12" s="11" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="G12" s="12">
+        <f>F12/$F$20</f>
+        <v/>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
         <is>
           <t>Bakers Authority (ADM Cornsweet)</t>
         </is>
@@ -1657,29 +1663,29 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>0.347</v>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
+        <v>0.33</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>$1.52 /lb</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="10" t="n">
         <v>1.52</v>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>50 lb</t>
         </is>
       </c>
-      <c r="F13" s="10" t="n">
-        <v>0.0012</v>
-      </c>
-      <c r="G13" s="11">
-        <f>F13/$F$19</f>
-        <v/>
-      </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="F13" s="11" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="G13" s="12">
+        <f>F13/$F$20</f>
+        <v/>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Internal: Complete Ingredients tab (Brenntag)</t>
         </is>
@@ -1688,33 +1694,33 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Ultra Masking Natural Flavor</t>
+          <t>Ultra Masking Nat 380223 (Gold Coast)</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.399</v>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
+        <v>0.38</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
-        <v>0.0074</v>
-      </c>
-      <c r="G14" s="11">
-        <f>F14/$F$19</f>
-        <v/>
-      </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="F14" s="11" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="G14" s="12">
+        <f>F14/$F$20</f>
+        <v/>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -1723,33 +1729,33 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Organic Lemon (flavor)</t>
+          <t>Organic Lemon 601032 (Gold Coast)</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.242</v>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
+        <v>0.23</v>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F15" s="10" t="n">
-        <v>0.0045</v>
-      </c>
-      <c r="G15" s="11">
-        <f>F15/$F$19</f>
-        <v/>
-      </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="F15" s="11" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="G15" s="12">
+        <f>F15/$F$20</f>
+        <v/>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -1758,33 +1764,33 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Natural Raspberry Flavor</t>
+          <t>Natural Raspberry Flavor 161443 (Gold Coast)</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>0.714</v>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
+        <v>0.68</v>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n">
-        <v>0.0132</v>
-      </c>
-      <c r="G16" s="11">
-        <f>F16/$F$19</f>
-        <v/>
-      </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="F16" s="11" t="n">
+        <v>0.0126</v>
+      </c>
+      <c r="G16" s="12">
+        <f>F16/$F$20</f>
+        <v/>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -1793,33 +1799,33 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Organic Cranberry Flavor</t>
+          <t>Organic Chamomile Flavor 357484 (Gold Coast)</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>0.368</v>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
+        <v>0.35</v>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F17" s="10" t="n">
-        <v>0.0068</v>
-      </c>
-      <c r="G17" s="11">
-        <f>F17/$F$19</f>
-        <v/>
-      </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="F17" s="11" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="G17" s="12">
+        <f>F17/$F$20</f>
+        <v/>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -1828,70 +1834,116 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Signature Beverage Enhancer</t>
+          <t>Organic Cranberry Flavor 606856 (Gold Coast)</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>0.714</v>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
+        <v>0.68</v>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>1 gal</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>0.0126</v>
+      </c>
+      <c r="G18" s="12">
+        <f>F18/$F$20</f>
+        <v/>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Signature Beverage Enhancer (Blue Pacific)</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
         <is>
           <t>$34.00 /lb</t>
         </is>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D19" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>1 lb</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n">
-        <v>0.0535</v>
-      </c>
-      <c r="G18" s="11">
-        <f>F18/$F$19</f>
-        <v/>
-      </c>
-      <c r="H18" s="12" t="inlineStr">
-        <is>
-          <t>Internal: Complete Ingredients tab (Signature Flavors analog)</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="F19" s="11" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="G19" s="12">
+        <f>F19/$F$20</f>
+        <v/>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Blue Pacific Flavors analog (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>TOTAL ingredient cost / can</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n"/>
-      <c r="C19" s="16" t="n"/>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="17">
-        <f>SUM(F5:F18)</f>
-        <v/>
-      </c>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Cost / 24-can case</t>
-        </is>
-      </c>
-      <c r="F20" s="19">
-        <f>F19*24</f>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="18">
+        <f>SUM(F5:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="17" t="n"/>
+      <c r="H20" s="17" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + 5% production-loss (purchasing basis)</t>
+        </is>
+      </c>
+      <c r="F21" s="20">
+        <f>F20*1.05</f>
         <v/>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>Orange = researched estimate (no firm internal/quoted price). Tighten with actual PO/invoice cost.</t>
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Cost / 12-pack (with loss)</t>
+        </is>
+      </c>
+      <c r="F22" s="22">
+        <f>F21*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>Orange = researched estimate (no firm internal/quoted price). Replace with actual PO cost to finalize.</t>
         </is>
       </c>
     </row>
@@ -1913,17 +1965,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H22"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1936,19 +1988,19 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>355 mL can | 24/case | 5% production-loss adj included | linear (marginal) ingredient cost, MOQ not loaded</t>
+          <t>250 mL fill | 12-pack | source: Spec tab (embedded image). Spec g/can are exact; cost = spec x cost/lb (no loss). Loss line below.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Ingredient</t>
+          <t>Ingredient (per spec)</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Amt/can (g)</t>
+          <t>Spec g/can</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -1958,7 +2010,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Cost/lb ($)</t>
+          <t>Cost/lb $</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -1968,12 +2020,12 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Cost/can ($)</t>
+          <t>Cost/can $</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>% of ing. cost</t>
+          <t>% ing.</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -1985,35 +2037,35 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Treated Water (RO)</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>360.861</v>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
+        <v>242</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>$0.10 /gal</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="10" t="n">
         <v>0.01</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F5" s="10" t="n">
-        <v>0.0095</v>
-      </c>
-      <c r="G5" s="11">
+      <c r="F5" s="11" t="n">
+        <v>0.0064</v>
+      </c>
+      <c r="G5" s="12">
         <f>F5/$F$19</f>
         <v/>
       </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>Internal: spec sheet (Drayhorse)</t>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Internal: spec sheet (Drayhorse RO)</t>
         </is>
       </c>
     </row>
@@ -2024,29 +2076,29 @@
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>0.112</v>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
+        <v>0.075</v>
+      </c>
+      <c r="C6" s="10" t="inlineStr">
         <is>
           <t>$4.82 /kg</t>
         </is>
       </c>
-      <c r="D6" s="9" t="n">
+      <c r="D6" s="10" t="n">
         <v>2.19</v>
       </c>
-      <c r="E6" s="9" t="inlineStr">
+      <c r="E6" s="10" t="inlineStr">
         <is>
           <t>~55 lb</t>
         </is>
       </c>
-      <c r="F6" s="10" t="n">
-        <v>0.0005</v>
-      </c>
-      <c r="G6" s="11">
+      <c r="F6" s="11" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="G6" s="12">
         <f>F6/$F$19</f>
         <v/>
       </c>
-      <c r="H6" s="12" t="inlineStr">
+      <c r="H6" s="13" t="inlineStr">
         <is>
           <t>Internal: Katana avg cost</t>
         </is>
@@ -2059,29 +2111,29 @@
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>0.112</v>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
+        <v>0.075</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
         <is>
           <t>$2.86 /kg</t>
         </is>
       </c>
-      <c r="D7" s="9" t="n">
+      <c r="D7" s="10" t="n">
         <v>1.3</v>
       </c>
-      <c r="E7" s="9" t="inlineStr">
+      <c r="E7" s="10" t="inlineStr">
         <is>
           <t>55 lb</t>
         </is>
       </c>
-      <c r="F7" s="10" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="G7" s="11">
+      <c r="F7" s="11" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="G7" s="12">
         <f>F7/$F$19</f>
         <v/>
       </c>
-      <c r="H7" s="12" t="inlineStr">
+      <c r="H7" s="13" t="inlineStr">
         <is>
           <t>Internal: Katana avg cost</t>
         </is>
@@ -2090,105 +2142,105 @@
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>Sodium Copper Chlorophyllin CVA</t>
+          <t>Sodium Copper Chlorophyllin CVA101808 (Naturex)</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>0.188</v>
-      </c>
-      <c r="C8" s="13" t="inlineStr">
+        <v>0.126</v>
+      </c>
+      <c r="C8" s="14" t="inlineStr">
         <is>
           <t>$60.00 /kg</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="14" t="n">
         <v>27.22</v>
       </c>
-      <c r="E8" s="9" t="inlineStr">
+      <c r="E8" s="10" t="inlineStr">
         <is>
           <t>1-25 kg</t>
         </is>
       </c>
-      <c r="F8" s="10" t="n">
-        <v>0.0113</v>
-      </c>
-      <c r="G8" s="11">
+      <c r="F8" s="11" t="n">
+        <v>0.0076</v>
+      </c>
+      <c r="G8" s="12">
         <f>F8/$F$19</f>
         <v/>
       </c>
-      <c r="H8" s="14" t="inlineStr">
-        <is>
-          <t>Nutri Avenue (E141 green color, est.)</t>
+      <c r="H8" s="15" t="inlineStr">
+        <is>
+          <t>Naturex / Nutri Avenue E141 (est.)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>CBD Hydrobond</t>
+          <t>CBD Hydrobond 685449</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>0.075</v>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
+        <v>0.05</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
         <is>
           <t>$300.00 /kg</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="14" t="n">
         <v>136.08</v>
       </c>
-      <c r="E9" s="9" t="inlineStr">
+      <c r="E9" s="10" t="inlineStr">
         <is>
           <t>1 kg</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n">
-        <v>0.0224</v>
-      </c>
-      <c r="G9" s="11">
+      <c r="F9" s="11" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G9" s="12">
         <f>F9/$F$19</f>
         <v/>
       </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>Hemp Depot (water-soluble CBD powder)</t>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>Hemp Depot water-soluble CBD (est.)</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="8" t="inlineStr">
         <is>
-          <t>Talin PG95</t>
+          <t>Talin PG95 T0001 (Naturex)</t>
         </is>
       </c>
       <c r="B10" s="9" t="n">
-        <v>0.522</v>
-      </c>
-      <c r="C10" s="13" t="inlineStr">
+        <v>0.35</v>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
         <is>
           <t>$200.00 /kg</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="14" t="n">
         <v>90.72</v>
       </c>
-      <c r="E10" s="9" t="inlineStr">
+      <c r="E10" s="10" t="inlineStr">
         <is>
           <t>1 kg</t>
         </is>
       </c>
-      <c r="F10" s="10" t="n">
-        <v>0.1044</v>
-      </c>
-      <c r="G10" s="11">
+      <c r="F10" s="11" t="n">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="G10" s="12">
         <f>F10/$F$19</f>
         <v/>
       </c>
-      <c r="H10" s="14" t="inlineStr">
-        <is>
-          <t>Knowde (Naturex/Givaudan Talin) + bulk thaumatin</t>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Naturex/Givaudan Talin; bulk thaumatin (est.)</t>
         </is>
       </c>
     </row>
@@ -2199,29 +2251,29 @@
         </is>
       </c>
       <c r="B11" s="9" t="n">
-        <v>1.491</v>
-      </c>
-      <c r="C11" s="13" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
         <is>
           <t>$1.20 /lb</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="14" t="n">
         <v>1.2</v>
       </c>
-      <c r="E11" s="9" t="inlineStr">
+      <c r="E11" s="10" t="inlineStr">
         <is>
           <t>50 lb</t>
         </is>
       </c>
-      <c r="F11" s="10" t="n">
-        <v>0.0039</v>
-      </c>
-      <c r="G11" s="11">
+      <c r="F11" s="11" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="G11" s="12">
         <f>F11/$F$19</f>
         <v/>
       </c>
-      <c r="H11" s="14" t="inlineStr">
+      <c r="H11" s="15" t="inlineStr">
         <is>
           <t>Bakers Authority (ADM Cornsweet)</t>
         </is>
@@ -2234,29 +2286,29 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>0.343</v>
-      </c>
-      <c r="C12" s="9" t="inlineStr">
+        <v>0.23</v>
+      </c>
+      <c r="C12" s="10" t="inlineStr">
         <is>
           <t>$1.52 /lb</t>
         </is>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="10" t="n">
         <v>1.52</v>
       </c>
-      <c r="E12" s="9" t="inlineStr">
+      <c r="E12" s="10" t="inlineStr">
         <is>
           <t>50 lb</t>
         </is>
       </c>
-      <c r="F12" s="10" t="n">
-        <v>0.0011</v>
-      </c>
-      <c r="G12" s="11">
+      <c r="F12" s="11" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="G12" s="12">
         <f>F12/$F$19</f>
         <v/>
       </c>
-      <c r="H12" s="12" t="inlineStr">
+      <c r="H12" s="13" t="inlineStr">
         <is>
           <t>Internal: Complete Ingredients tab (Brenntag)</t>
         </is>
@@ -2265,33 +2317,33 @@
     <row r="13">
       <c r="A13" s="8" t="inlineStr">
         <is>
-          <t>Ultra Masking Natural Flavor</t>
+          <t>Ultra Masking Nat 380223 (Gold Coast)</t>
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>1.193</v>
-      </c>
-      <c r="C13" s="9" t="inlineStr">
+        <v>0.8</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D13" s="9" t="n">
+      <c r="D13" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E13" s="9" t="inlineStr">
+      <c r="E13" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F13" s="10" t="n">
-        <v>0.0221</v>
-      </c>
-      <c r="G13" s="11">
+      <c r="F13" s="11" t="n">
+        <v>0.0148</v>
+      </c>
+      <c r="G13" s="12">
         <f>F13/$F$19</f>
         <v/>
       </c>
-      <c r="H13" s="12" t="inlineStr">
+      <c r="H13" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -2300,33 +2352,33 @@
     <row r="14">
       <c r="A14" s="8" t="inlineStr">
         <is>
-          <t>Organic Cranberry Flavor</t>
+          <t>Organic Cranberry Flavor 606856 (Gold Coast)</t>
         </is>
       </c>
       <c r="B14" s="9" t="n">
-        <v>0.895</v>
-      </c>
-      <c r="C14" s="9" t="inlineStr">
+        <v>0.6</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D14" s="9" t="n">
+      <c r="D14" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E14" s="9" t="inlineStr">
+      <c r="E14" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F14" s="10" t="n">
-        <v>0.0165</v>
-      </c>
-      <c r="G14" s="11">
+      <c r="F14" s="11" t="n">
+        <v>0.0111</v>
+      </c>
+      <c r="G14" s="12">
         <f>F14/$F$19</f>
         <v/>
       </c>
-      <c r="H14" s="12" t="inlineStr">
+      <c r="H14" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -2335,33 +2387,33 @@
     <row r="15">
       <c r="A15" s="8" t="inlineStr">
         <is>
-          <t>Organic Lime Flavor</t>
+          <t>Organic Lime Flavor 309465 (Gold Coast)</t>
         </is>
       </c>
       <c r="B15" s="9" t="n">
-        <v>0.142</v>
-      </c>
-      <c r="C15" s="9" t="inlineStr">
+        <v>0.095</v>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D15" s="9" t="n">
+      <c r="D15" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E15" s="9" t="inlineStr">
+      <c r="E15" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F15" s="10" t="n">
-        <v>0.0026</v>
-      </c>
-      <c r="G15" s="11">
+      <c r="F15" s="11" t="n">
+        <v>0.0018</v>
+      </c>
+      <c r="G15" s="12">
         <f>F15/$F$19</f>
         <v/>
       </c>
-      <c r="H15" s="12" t="inlineStr">
+      <c r="H15" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -2370,33 +2422,33 @@
     <row r="16">
       <c r="A16" s="8" t="inlineStr">
         <is>
-          <t>Natural Cucumber Flavor</t>
+          <t>Natural Cucumber Flavor 336018 (Gold Coast)</t>
         </is>
       </c>
       <c r="B16" s="9" t="n">
-        <v>0.358</v>
-      </c>
-      <c r="C16" s="9" t="inlineStr">
+        <v>0.24</v>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D16" s="9" t="n">
+      <c r="D16" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E16" s="9" t="inlineStr">
+      <c r="E16" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F16" s="10" t="n">
-        <v>0.0066</v>
-      </c>
-      <c r="G16" s="11">
+      <c r="F16" s="11" t="n">
+        <v>0.0044</v>
+      </c>
+      <c r="G16" s="12">
         <f>F16/$F$19</f>
         <v/>
       </c>
-      <c r="H16" s="12" t="inlineStr">
+      <c r="H16" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -2405,33 +2457,33 @@
     <row r="17">
       <c r="A17" s="8" t="inlineStr">
         <is>
-          <t>Natural Cucumber</t>
+          <t>Natural Cucumber S1511015 (FONA)</t>
         </is>
       </c>
       <c r="B17" s="9" t="n">
-        <v>0.716</v>
-      </c>
-      <c r="C17" s="9" t="inlineStr">
+        <v>0.48</v>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
         <is>
           <t>$70.00 /gal</t>
         </is>
       </c>
-      <c r="D17" s="9" t="n">
+      <c r="D17" s="10" t="n">
         <v>8.390000000000001</v>
       </c>
-      <c r="E17" s="9" t="inlineStr">
+      <c r="E17" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F17" s="10" t="n">
-        <v>0.0132</v>
-      </c>
-      <c r="G17" s="11">
+      <c r="F17" s="11" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="G17" s="12">
         <f>F17/$F$19</f>
         <v/>
       </c>
-      <c r="H17" s="12" t="inlineStr">
+      <c r="H17" s="13" t="inlineStr">
         <is>
           <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
         </is>
@@ -2440,70 +2492,81 @@
     <row r="18">
       <c r="A18" s="8" t="inlineStr">
         <is>
-          <t>Signature Beverage Enhancer</t>
+          <t>Signature Beverage Enhancer (Blue Pacific)</t>
         </is>
       </c>
       <c r="B18" s="9" t="n">
-        <v>0.119</v>
-      </c>
-      <c r="C18" s="13" t="inlineStr">
+        <v>0.08</v>
+      </c>
+      <c r="C18" s="14" t="inlineStr">
         <is>
           <t>$34.00 /lb</t>
         </is>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="14" t="n">
         <v>34</v>
       </c>
-      <c r="E18" s="9" t="inlineStr">
+      <c r="E18" s="10" t="inlineStr">
         <is>
           <t>1 lb</t>
         </is>
       </c>
-      <c r="F18" s="10" t="n">
-        <v>0.0089</v>
-      </c>
-      <c r="G18" s="11">
+      <c r="F18" s="11" t="n">
+        <v>0.006</v>
+      </c>
+      <c r="G18" s="12">
         <f>F18/$F$19</f>
         <v/>
       </c>
-      <c r="H18" s="12" t="inlineStr">
-        <is>
-          <t>Internal: Complete Ingredients tab (Signature Flavors analog)</t>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Blue Pacific Flavors analog (est.)</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="15" t="inlineStr">
+      <c r="A19" s="16" t="inlineStr">
         <is>
           <t>TOTAL ingredient cost / can</t>
         </is>
       </c>
-      <c r="B19" s="16" t="n"/>
-      <c r="C19" s="16" t="n"/>
-      <c r="D19" s="16" t="n"/>
-      <c r="E19" s="16" t="n"/>
-      <c r="F19" s="17">
+      <c r="B19" s="17" t="n"/>
+      <c r="C19" s="17" t="n"/>
+      <c r="D19" s="17" t="n"/>
+      <c r="E19" s="17" t="n"/>
+      <c r="F19" s="18">
         <f>SUM(F5:F18)</f>
         <v/>
       </c>
-      <c r="G19" s="16" t="n"/>
-      <c r="H19" s="16" t="n"/>
+      <c r="G19" s="17" t="n"/>
+      <c r="H19" s="17" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="18" t="inlineStr">
-        <is>
-          <t>Cost / 24-can case</t>
-        </is>
-      </c>
-      <c r="F20" s="19">
-        <f>F19*24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" s="20" t="inlineStr">
-        <is>
-          <t>Orange = researched estimate (no firm internal/quoted price). Tighten with actual PO/invoice cost.</t>
+      <c r="A20" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + 5% production-loss (purchasing basis)</t>
+        </is>
+      </c>
+      <c r="F20" s="20">
+        <f>F19*1.05</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="21" t="inlineStr">
+        <is>
+          <t>Cost / 12-pack (with loss)</t>
+        </is>
+      </c>
+      <c r="F21" s="22">
+        <f>F20*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="23" t="inlineStr">
+        <is>
+          <t>Orange = researched estimate (no firm internal/quoted price). Replace with actual PO cost to finalize.</t>
         </is>
       </c>
     </row>
@@ -2524,17 +2587,17 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
     <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="52" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2547,19 +2610,19 @@
     <row r="2">
       <c r="A2" s="6" t="inlineStr">
         <is>
-          <t>355 mL can | 24/case | 5% production-loss adj included | linear (marginal) ingredient cost, MOQ not loaded</t>
+          <t>250 mL fill | 12-pack | source: Spec tab (embedded image). Spec g/can are exact; cost = spec x cost/lb (no loss). Loss line below.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>Ingredient</t>
+          <t>Ingredient (per spec)</t>
         </is>
       </c>
       <c r="B4" s="7" t="inlineStr">
         <is>
-          <t>Amt/can (g)</t>
+          <t>Spec g/can</t>
         </is>
       </c>
       <c r="C4" s="7" t="inlineStr">
@@ -2569,7 +2632,7 @@
       </c>
       <c r="D4" s="7" t="inlineStr">
         <is>
-          <t>Cost/lb ($)</t>
+          <t>Cost/lb $</t>
         </is>
       </c>
       <c r="E4" s="7" t="inlineStr">
@@ -2579,12 +2642,12 @@
       </c>
       <c r="F4" s="7" t="inlineStr">
         <is>
-          <t>Cost/can ($)</t>
+          <t>Cost/can $</t>
         </is>
       </c>
       <c r="G4" s="7" t="inlineStr">
         <is>
-          <t>% of ing. cost</t>
+          <t>% ing.</t>
         </is>
       </c>
       <c r="H4" s="7" t="inlineStr">
@@ -2596,216 +2659,581 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>Water</t>
+          <t>Treated Water (RO)</t>
         </is>
       </c>
       <c r="B5" s="9" t="n">
-        <v>325.44</v>
-      </c>
-      <c r="C5" s="9" t="inlineStr">
+        <v>233.2</v>
+      </c>
+      <c r="C5" s="10" t="inlineStr">
         <is>
           <t>$0.10 /gal</t>
         </is>
       </c>
-      <c r="D5" s="9" t="n">
+      <c r="D5" s="10" t="n">
         <v>0.01</v>
       </c>
-      <c r="E5" s="9" t="inlineStr">
+      <c r="E5" s="10" t="inlineStr">
         <is>
           <t>1 gal</t>
         </is>
       </c>
-      <c r="F5" s="10" t="n">
-        <v>0.0086</v>
-      </c>
-      <c r="G5" s="11">
-        <f>F5/$F$10</f>
-        <v/>
-      </c>
-      <c r="H5" s="12" t="inlineStr">
-        <is>
-          <t>Internal: spec sheet (Drayhorse)</t>
+      <c r="F5" s="11" t="n">
+        <v>0.0062</v>
+      </c>
+      <c r="G5" s="12">
+        <f>F5/$F$20</f>
+        <v/>
+      </c>
+      <c r="H5" s="13" t="inlineStr">
+        <is>
+          <t>Internal: spec sheet (Drayhorse RO)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>GNS (45%)</t>
+          <t>Vegetable Glycerin (Cacee)</t>
         </is>
       </c>
       <c r="B6" s="9" t="n">
-        <v>41.992</v>
-      </c>
-      <c r="C6" s="9" t="inlineStr">
-        <is>
-          <t>$5.56 /gal</t>
-        </is>
-      </c>
-      <c r="D6" s="9" t="n">
-        <v>0.78</v>
-      </c>
-      <c r="E6" s="9" t="inlineStr">
-        <is>
-          <t>275 gal</t>
-        </is>
-      </c>
-      <c r="F6" s="10" t="n">
-        <v>0.0726</v>
-      </c>
-      <c r="G6" s="11">
-        <f>F6/$F$10</f>
-        <v/>
-      </c>
-      <c r="H6" s="12" t="inlineStr">
-        <is>
-          <t>Internal: Complete Ingredients tab (GNS 95%, Brooklyn/Ultrapure)</t>
+        <v>12.1</v>
+      </c>
+      <c r="C6" s="14" t="inlineStr">
+        <is>
+          <t>$2.00 /lb</t>
+        </is>
+      </c>
+      <c r="D6" s="14" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" s="10" t="inlineStr">
+        <is>
+          <t>50 lb</t>
+        </is>
+      </c>
+      <c r="F6" s="11" t="n">
+        <v>0.0534</v>
+      </c>
+      <c r="G6" s="12">
+        <f>F6/$F$20</f>
+        <v/>
+      </c>
+      <c r="H6" s="15" t="inlineStr">
+        <is>
+          <t>Bulk Apothecary / Jedwards (USP, est.)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>Lemon Juice Concentrate</t>
+          <t>Potassium Benzoate</t>
         </is>
       </c>
       <c r="B7" s="9" t="n">
-        <v>5.249</v>
-      </c>
-      <c r="C7" s="9" t="inlineStr">
-        <is>
-          <t>$2.91 /lb</t>
-        </is>
-      </c>
-      <c r="D7" s="9" t="n">
-        <v>2.91</v>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>51 lb</t>
-        </is>
-      </c>
-      <c r="F7" s="10" t="n">
-        <v>0.0337</v>
-      </c>
-      <c r="G7" s="11">
-        <f>F7/$F$10</f>
-        <v/>
-      </c>
-      <c r="H7" s="12" t="inlineStr">
-        <is>
-          <t>Internal: Complete Ingredients tab (Greenwood)</t>
+        <v>0.075</v>
+      </c>
+      <c r="C7" s="10" t="inlineStr">
+        <is>
+          <t>$4.82 /kg</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="E7" s="10" t="inlineStr">
+        <is>
+          <t>~55 lb</t>
+        </is>
+      </c>
+      <c r="F7" s="11" t="n">
+        <v>0.0004</v>
+      </c>
+      <c r="G7" s="12">
+        <f>F7/$F$20</f>
+        <v/>
+      </c>
+      <c r="H7" s="13" t="inlineStr">
+        <is>
+          <t>Internal: Katana avg cost</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="8" t="inlineStr">
         <is>
-          <t>White Cane Sugar</t>
+          <t>Potassium Sorbate</t>
         </is>
       </c>
       <c r="B8" s="9" t="n">
-        <v>5.249</v>
-      </c>
-      <c r="C8" s="9" t="inlineStr">
-        <is>
-          <t>$0.94 /lb</t>
-        </is>
-      </c>
-      <c r="D8" s="9" t="n">
-        <v>0.9399999999999999</v>
-      </c>
-      <c r="E8" s="9" t="inlineStr">
-        <is>
-          <t>50 lb</t>
-        </is>
-      </c>
-      <c r="F8" s="10" t="n">
-        <v>0.0109</v>
-      </c>
-      <c r="G8" s="11">
-        <f>F8/$F$10</f>
-        <v/>
-      </c>
-      <c r="H8" s="12" t="inlineStr">
-        <is>
-          <t>Internal: Complete Ingredients tab (Granulated Sugar)</t>
+        <v>0.075</v>
+      </c>
+      <c r="C8" s="10" t="inlineStr">
+        <is>
+          <t>$2.86 /kg</t>
+        </is>
+      </c>
+      <c r="D8" s="10" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="E8" s="10" t="inlineStr">
+        <is>
+          <t>55 lb</t>
+        </is>
+      </c>
+      <c r="F8" s="11" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="G8" s="12">
+        <f>F8/$F$20</f>
+        <v/>
+      </c>
+      <c r="H8" s="13" t="inlineStr">
+        <is>
+          <t>Internal: Katana avg cost</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="8" t="inlineStr">
         <is>
-          <t>Lemon Verbena Cut &amp; Sifted</t>
+          <t>Sodium Copper Chlorophyllin CA101808 (Naturex)</t>
         </is>
       </c>
       <c r="B9" s="9" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="C9" s="13" t="inlineStr">
-        <is>
-          <t>$12.00 /lb</t>
-        </is>
-      </c>
-      <c r="D9" s="13" t="n">
-        <v>12</v>
-      </c>
-      <c r="E9" s="9" t="inlineStr">
+        <v>0.246</v>
+      </c>
+      <c r="C9" s="14" t="inlineStr">
+        <is>
+          <t>$60.00 /kg</t>
+        </is>
+      </c>
+      <c r="D9" s="14" t="n">
+        <v>27.22</v>
+      </c>
+      <c r="E9" s="10" t="inlineStr">
+        <is>
+          <t>1-25 kg</t>
+        </is>
+      </c>
+      <c r="F9" s="11" t="n">
+        <v>0.0148</v>
+      </c>
+      <c r="G9" s="12">
+        <f>F9/$F$20</f>
+        <v/>
+      </c>
+      <c r="H9" s="15" t="inlineStr">
+        <is>
+          <t>Naturex / Nutri Avenue E141 (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>CBD Hydrobond 685449</t>
+        </is>
+      </c>
+      <c r="B10" s="9" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C10" s="14" t="inlineStr">
+        <is>
+          <t>$300.00 /kg</t>
+        </is>
+      </c>
+      <c r="D10" s="14" t="n">
+        <v>136.08</v>
+      </c>
+      <c r="E10" s="10" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
+      <c r="F10" s="11" t="n">
+        <v>0.015</v>
+      </c>
+      <c r="G10" s="12">
+        <f>F10/$F$20</f>
+        <v/>
+      </c>
+      <c r="H10" s="15" t="inlineStr">
+        <is>
+          <t>Hemp Depot water-soluble CBD (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Talin PG95 T0001 (Naturex)</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>$200.00 /kg</t>
+        </is>
+      </c>
+      <c r="D11" s="14" t="n">
+        <v>90.72</v>
+      </c>
+      <c r="E11" s="10" t="inlineStr">
+        <is>
+          <t>1 kg</t>
+        </is>
+      </c>
+      <c r="F11" s="11" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="G11" s="12">
+        <f>F11/$F$20</f>
+        <v/>
+      </c>
+      <c r="H11" s="15" t="inlineStr">
+        <is>
+          <t>Naturex/Givaudan Talin; bulk thaumatin (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Crystalline Fructose</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>1</v>
+      </c>
+      <c r="C12" s="14" t="inlineStr">
+        <is>
+          <t>$1.20 /lb</t>
+        </is>
+      </c>
+      <c r="D12" s="14" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="E12" s="10" t="inlineStr">
+        <is>
+          <t>50 lb</t>
+        </is>
+      </c>
+      <c r="F12" s="11" t="n">
+        <v>0.0026</v>
+      </c>
+      <c r="G12" s="12">
+        <f>F12/$F$20</f>
+        <v/>
+      </c>
+      <c r="H12" s="15" t="inlineStr">
+        <is>
+          <t>Bakers Authority (ADM Cornsweet)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Citric Acid</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C13" s="10" t="inlineStr">
+        <is>
+          <t>$1.52 /lb</t>
+        </is>
+      </c>
+      <c r="D13" s="10" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="E13" s="10" t="inlineStr">
+        <is>
+          <t>50 lb</t>
+        </is>
+      </c>
+      <c r="F13" s="11" t="n">
+        <v>0.0005</v>
+      </c>
+      <c r="G13" s="12">
+        <f>F13/$F$20</f>
+        <v/>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>Internal: Complete Ingredients tab (Brenntag)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Ultra Masking Nat 380223 (Gold Coast)</t>
+        </is>
+      </c>
+      <c r="B14" s="9" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="C14" s="10" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D14" s="10" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="E14" s="10" t="inlineStr">
+        <is>
+          <t>1 gal</t>
+        </is>
+      </c>
+      <c r="F14" s="11" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="G14" s="12">
+        <f>F14/$F$20</f>
+        <v/>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Organic Lemon 601032 (Gold Coast)</t>
+        </is>
+      </c>
+      <c r="B15" s="9" t="n">
+        <v>0.23</v>
+      </c>
+      <c r="C15" s="10" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D15" s="10" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="E15" s="10" t="inlineStr">
+        <is>
+          <t>1 gal</t>
+        </is>
+      </c>
+      <c r="F15" s="11" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="G15" s="12">
+        <f>F15/$F$20</f>
+        <v/>
+      </c>
+      <c r="H15" s="13" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Organic Lime 309465 (Gold Coast)</t>
+        </is>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>0.28</v>
+      </c>
+      <c r="C16" s="10" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D16" s="10" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="E16" s="10" t="inlineStr">
+        <is>
+          <t>1 gal</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="n">
+        <v>0.0052</v>
+      </c>
+      <c r="G16" s="12">
+        <f>F16/$F$20</f>
+        <v/>
+      </c>
+      <c r="H16" s="13" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Natural Bergamot Flavor (Gold Coast)</t>
+        </is>
+      </c>
+      <c r="B17" s="9" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="C17" s="10" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D17" s="10" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="E17" s="10" t="inlineStr">
+        <is>
+          <t>1 gal</t>
+        </is>
+      </c>
+      <c r="F17" s="11" t="n">
+        <v>0.0065</v>
+      </c>
+      <c r="G17" s="12">
+        <f>F17/$F$20</f>
+        <v/>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>Organic Cranberry Flavor 606856 (Gold Coast)</t>
+        </is>
+      </c>
+      <c r="B18" s="9" t="n">
+        <v>0.38</v>
+      </c>
+      <c r="C18" s="10" t="inlineStr">
+        <is>
+          <t>$70.00 /gal</t>
+        </is>
+      </c>
+      <c r="D18" s="10" t="n">
+        <v>8.390000000000001</v>
+      </c>
+      <c r="E18" s="10" t="inlineStr">
+        <is>
+          <t>1 gal</t>
+        </is>
+      </c>
+      <c r="F18" s="11" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="G18" s="12">
+        <f>F18/$F$20</f>
+        <v/>
+      </c>
+      <c r="H18" s="13" t="inlineStr">
+        <is>
+          <t>Client-directed: $70/gal (SG 1.0 assumed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>Signature Beverage Enhancer (Blue Pacific)</t>
+        </is>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>$34.00 /lb</t>
+        </is>
+      </c>
+      <c r="D19" s="14" t="n">
+        <v>34</v>
+      </c>
+      <c r="E19" s="10" t="inlineStr">
         <is>
           <t>1 lb</t>
         </is>
       </c>
-      <c r="F9" s="10" t="n">
-        <v>0.0555</v>
-      </c>
-      <c r="G9" s="11">
-        <f>F9/$F$10</f>
-        <v/>
-      </c>
-      <c r="H9" s="14" t="inlineStr">
-        <is>
-          <t>Monterey Bay Herb Co (est.)</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="15" t="inlineStr">
+      <c r="F19" s="11" t="n">
+        <v>0.008999999999999999</v>
+      </c>
+      <c r="G19" s="12">
+        <f>F19/$F$20</f>
+        <v/>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>Blue Pacific Flavors analog (est.)</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="16" t="inlineStr">
         <is>
           <t>TOTAL ingredient cost / can</t>
         </is>
       </c>
-      <c r="B10" s="16" t="n"/>
-      <c r="C10" s="16" t="n"/>
-      <c r="D10" s="16" t="n"/>
-      <c r="E10" s="16" t="n"/>
-      <c r="F10" s="17">
-        <f>SUM(F5:F9)</f>
-        <v/>
-      </c>
-      <c r="G10" s="16" t="n"/>
-      <c r="H10" s="16" t="n"/>
-    </row>
-    <row r="11">
-      <c r="A11" s="18" t="inlineStr">
-        <is>
-          <t>Cost / 24-can case</t>
-        </is>
-      </c>
-      <c r="F11" s="19">
-        <f>F10*24</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="20" t="inlineStr">
-        <is>
-          <t>Orange = researched estimate (no firm internal/quoted price). Tighten with actual PO/invoice cost.</t>
+      <c r="B20" s="17" t="n"/>
+      <c r="C20" s="17" t="n"/>
+      <c r="D20" s="17" t="n"/>
+      <c r="E20" s="17" t="n"/>
+      <c r="F20" s="18">
+        <f>SUM(F5:F19)</f>
+        <v/>
+      </c>
+      <c r="G20" s="17" t="n"/>
+      <c r="H20" s="17" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  + 5% production-loss (purchasing basis)</t>
+        </is>
+      </c>
+      <c r="F21" s="20">
+        <f>F20*1.05</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="21" t="inlineStr">
+        <is>
+          <t>Cost / 12-pack (with loss)</t>
+        </is>
+      </c>
+      <c r="F22" s="22">
+        <f>F21*12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="23" t="inlineStr">
+        <is>
+          <t>Orange = researched estimate (no firm internal/quoted price). Replace with actual PO cost to finalize.</t>
         </is>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H6" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H9" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H10" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H11" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="H12" r:id="rId5"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Source food-grade chamomile hydrosol; cost by spec volume
Chamomile must stay a hydrosol (no hot brew), so the line now points at
genuinely food-grade bulk suppliers (Florihana edible / Shay & Co / Organic
Creations, quote pending) and is costed by its spec volume (19.04 mL/can)
rather than mass, since hydrosol is sold by volume. Flags the ~$40-90/gal
range for organic German chamomile.

https://claude.ai/code/session_01Xys6L7LsgSa2ACDzAaru9U
</commit_message>
<xml_diff>
--- a/STH_Run001_Ingredient_Cost_Per_Can.xlsx
+++ b/STH_Run001_Ingredient_Cost_Per_Can.xlsx
@@ -655,21 +655,21 @@
     <row r="21">
       <c r="A21" s="3" t="inlineStr">
         <is>
-          <t>Orange cells = researched estimates (CBD Hydrobond, Talin PG95, natural colors, chamomile hydrosol, vegetable glycerin,</t>
+          <t>Orange cells = researched estimates. Chamomile hydrosol must be FOOD-GRADE (most aromatherapy hydrosols are cosmetic-only);</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>Signature Enhancer). Biggest swing factors: Serenity chamomile hydrosol (~$0.22/can) and Talin. Firm: water, citric acid,</t>
+          <t>costed by spec volume (19.04 mL/can) at ~$50/gal placeholder - get a firm quote + COA (organic German runs $40-90/gal).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>fructose, preservatives, Bossen lychee. Replace orange items with actual purchase costs to finalize.</t>
+          <t>Other orange items: CBD Hydrobond, Talin PG95, colors, vegetable glycerin. Firm: water, citric acid, fructose, preservatives, Bossen lychee.</t>
         </is>
       </c>
     </row>
@@ -1426,15 +1426,15 @@
         </is>
       </c>
       <c r="D6" s="14" t="n">
-        <v>5.99</v>
+        <v>6.79</v>
       </c>
       <c r="E6" s="10" t="inlineStr">
         <is>
-          <t>1 gal</t>
+          <t>5 gal / drum</t>
         </is>
       </c>
       <c r="F6" s="11" t="n">
-        <v>0.2219</v>
+        <v>0.2516</v>
       </c>
       <c r="G6" s="12">
         <f>F6/$F$20</f>
@@ -1442,7 +1442,7 @@
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>Mountain Rose Herbs (est.)</t>
+          <t>Food-grade organic hydrosol: Florihana (edible) / Shay &amp; Co / Organic Creations - quote pending (~$40-90/gal organic German)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Express recipe amounts in lbs across all formulas
RECIPE UNIT is now lbs for every ingredient at the 100-gal base batch;
BUY UNIT stays per-ingredient (gal/lbs/kg). SG converts lbs->gal for the
volume-bought liquids. Run scale-up need shown in lbs, purchase qty in buy
unit. Costs unchanged.

https://claude.ai/code/session_01Xys6L7LsgSa2ACDzAaru9U
</commit_message>
<xml_diff>
--- a/STH_Run001_Ingredient_Cost_Per_Can.xlsx
+++ b/STH_Run001_Ingredient_Cost_Per_Can.xlsx
@@ -744,12 +744,12 @@
       </c>
       <c r="K1" s="9" t="inlineStr">
         <is>
-          <t>NEED /2000 cases (+5% loss)</t>
+          <t>NEED /2000 cases (lbs,+5% loss)</t>
         </is>
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>BUY QTY (MOQ-adj)</t>
+          <t>BUY QTY (MOQ-adj, buy unit)</t>
         </is>
       </c>
       <c r="M1" s="9" t="inlineStr">
@@ -770,11 +770,11 @@
         </is>
       </c>
       <c r="C2" s="10" t="n">
-        <v>98</v>
+        <v>817.8504</v>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E2" s="10" t="n">
@@ -796,7 +796,7 @@
       </c>
       <c r="J2" s="11" t="inlineStr"/>
       <c r="K2" s="10" t="n">
-        <v>1630.9982</v>
+        <v>13611.3512</v>
       </c>
       <c r="L2" s="10" t="n">
         <v>1631</v>
@@ -817,11 +817,11 @@
         </is>
       </c>
       <c r="C3" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.2504</v>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E3" s="10" t="n">
@@ -843,7 +843,7 @@
       </c>
       <c r="J3" s="11" t="inlineStr"/>
       <c r="K3" s="10" t="n">
-        <v>1.89</v>
+        <v>4.1667</v>
       </c>
       <c r="L3" s="10" t="n">
         <v>55</v>
@@ -864,11 +864,11 @@
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.2504</v>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E4" s="10" t="n">
@@ -890,7 +890,7 @@
       </c>
       <c r="J4" s="11" t="inlineStr"/>
       <c r="K4" s="10" t="n">
-        <v>1.89</v>
+        <v>4.1667</v>
       </c>
       <c r="L4" s="10" t="n">
         <v>55</v>
@@ -911,11 +911,11 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>0.1908</v>
+        <v>0.4206</v>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E5" s="10" t="n">
@@ -937,7 +937,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr"/>
       <c r="K5" s="10" t="n">
-        <v>3.1752</v>
+        <v>7.0001</v>
       </c>
       <c r="L5" s="10" t="n">
         <v>25</v>
@@ -958,11 +958,11 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>0.0757</v>
+        <v>0.1669</v>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E6" s="10" t="n">
@@ -984,7 +984,7 @@
       </c>
       <c r="J6" s="11" t="inlineStr"/>
       <c r="K6" s="10" t="n">
-        <v>1.26</v>
+        <v>2.7778</v>
       </c>
       <c r="L6" s="10" t="n">
         <v>2</v>
@@ -1052,11 +1052,11 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>0.53</v>
+        <v>1.1684</v>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E8" s="10" t="n">
@@ -1078,7 +1078,7 @@
       </c>
       <c r="J8" s="11" t="inlineStr"/>
       <c r="K8" s="10" t="n">
-        <v>8.82</v>
+        <v>19.4448</v>
       </c>
       <c r="L8" s="10" t="n">
         <v>9</v>
@@ -1193,11 +1193,11 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.152</v>
+        <v>1.2685</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E11" s="10" t="n">
@@ -1219,7 +1219,7 @@
       </c>
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="10" t="n">
-        <v>2.5297</v>
+        <v>21.1115</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>3</v>
@@ -1240,11 +1240,11 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>0.22</v>
+        <v>1.836</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
@@ -1266,7 +1266,7 @@
       </c>
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="10" t="n">
-        <v>3.6614</v>
+        <v>30.5561</v>
       </c>
       <c r="L12" s="10" t="n">
         <v>4</v>
@@ -1287,11 +1287,11 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>0.06</v>
+        <v>0.5007</v>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E13" s="10" t="n">
@@ -1313,7 +1313,7 @@
       </c>
       <c r="J13" s="11" t="inlineStr"/>
       <c r="K13" s="10" t="n">
-        <v>0.9986</v>
+        <v>8.333500000000001</v>
       </c>
       <c r="L13" s="10" t="n">
         <v>1</v>
@@ -1334,11 +1334,11 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>0.192</v>
+        <v>1.6023</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E14" s="10" t="n">
@@ -1360,7 +1360,7 @@
       </c>
       <c r="J14" s="11" t="inlineStr"/>
       <c r="K14" s="10" t="n">
-        <v>3.1954</v>
+        <v>26.6671</v>
       </c>
       <c r="L14" s="10" t="n">
         <v>4</v>
@@ -1517,12 +1517,12 @@
       </c>
       <c r="K1" s="9" t="inlineStr">
         <is>
-          <t>NEED /2000 cases (+5% loss)</t>
+          <t>NEED /2000 cases (lbs,+5% loss)</t>
         </is>
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>BUY QTY (MOQ-adj)</t>
+          <t>BUY QTY (MOQ-adj, buy unit)</t>
         </is>
       </c>
       <c r="M1" s="9" t="inlineStr">
@@ -1543,11 +1543,11 @@
         </is>
       </c>
       <c r="C2" s="10" t="n">
-        <v>90.88</v>
+        <v>758.431</v>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E2" s="10" t="n">
@@ -1569,7 +1569,7 @@
       </c>
       <c r="J2" s="11" t="inlineStr"/>
       <c r="K2" s="10" t="n">
-        <v>1512.5011</v>
+        <v>12622.4448</v>
       </c>
       <c r="L2" s="10" t="n">
         <v>1513</v>
@@ -1590,11 +1590,11 @@
         </is>
       </c>
       <c r="C3" s="10" t="n">
-        <v>6.72</v>
+        <v>56.0812</v>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E3" s="10" t="n">
@@ -1616,7 +1616,7 @@
       </c>
       <c r="J3" s="11" t="inlineStr"/>
       <c r="K3" s="10" t="n">
-        <v>111.8399</v>
+        <v>933.3498</v>
       </c>
       <c r="L3" s="10" t="n">
         <v>115</v>
@@ -1637,11 +1637,11 @@
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.2504</v>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E4" s="10" t="n">
@@ -1663,7 +1663,7 @@
       </c>
       <c r="J4" s="11" t="inlineStr"/>
       <c r="K4" s="10" t="n">
-        <v>1.89</v>
+        <v>4.1667</v>
       </c>
       <c r="L4" s="10" t="n">
         <v>55</v>
@@ -1684,11 +1684,11 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.2504</v>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E5" s="10" t="n">
@@ -1710,7 +1710,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr"/>
       <c r="K5" s="10" t="n">
-        <v>1.89</v>
+        <v>4.1667</v>
       </c>
       <c r="L5" s="10" t="n">
         <v>55</v>
@@ -1731,11 +1731,11 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>0.3422</v>
+        <v>0.7544</v>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E6" s="10" t="n">
@@ -1757,7 +1757,7 @@
       </c>
       <c r="J6" s="11" t="inlineStr"/>
       <c r="K6" s="10" t="n">
-        <v>5.6952</v>
+        <v>12.5558</v>
       </c>
       <c r="L6" s="10" t="n">
         <v>25</v>
@@ -1778,11 +1778,11 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.0757</v>
+        <v>0.1669</v>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E7" s="10" t="n">
@@ -1804,7 +1804,7 @@
       </c>
       <c r="J7" s="11" t="inlineStr"/>
       <c r="K7" s="10" t="n">
-        <v>1.26</v>
+        <v>2.7778</v>
       </c>
       <c r="L7" s="10" t="n">
         <v>2</v>
@@ -1825,11 +1825,11 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>0.6814</v>
+        <v>1.5022</v>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E8" s="10" t="n">
@@ -1851,7 +1851,7 @@
       </c>
       <c r="J8" s="11" t="inlineStr"/>
       <c r="K8" s="10" t="n">
-        <v>11.34</v>
+        <v>25.0004</v>
       </c>
       <c r="L8" s="10" t="n">
         <v>12</v>
@@ -1966,11 +1966,11 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.152</v>
+        <v>1.2685</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E11" s="10" t="n">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="10" t="n">
-        <v>2.5297</v>
+        <v>21.1115</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>3</v>
@@ -2013,11 +2013,11 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>0.092</v>
+        <v>0.7678</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
@@ -2039,7 +2039,7 @@
       </c>
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="10" t="n">
-        <v>1.5311</v>
+        <v>12.778</v>
       </c>
       <c r="L12" s="10" t="n">
         <v>2</v>
@@ -2060,11 +2060,11 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>0.272</v>
+        <v>2.27</v>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E13" s="10" t="n">
@@ -2086,7 +2086,7 @@
       </c>
       <c r="J13" s="11" t="inlineStr"/>
       <c r="K13" s="10" t="n">
-        <v>4.5269</v>
+        <v>37.7784</v>
       </c>
       <c r="L13" s="10" t="n">
         <v>5</v>
@@ -2107,11 +2107,11 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>0.14</v>
+        <v>1.1684</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E14" s="10" t="n">
@@ -2133,7 +2133,7 @@
       </c>
       <c r="J14" s="11" t="inlineStr"/>
       <c r="K14" s="10" t="n">
-        <v>2.33</v>
+        <v>19.4448</v>
       </c>
       <c r="L14" s="10" t="n">
         <v>3</v>
@@ -2154,11 +2154,11 @@
         </is>
       </c>
       <c r="C15" s="10" t="n">
-        <v>0.272</v>
+        <v>2.27</v>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E15" s="10" t="n">
@@ -2180,7 +2180,7 @@
       </c>
       <c r="J15" s="11" t="inlineStr"/>
       <c r="K15" s="10" t="n">
-        <v>4.5269</v>
+        <v>37.7784</v>
       </c>
       <c r="L15" s="10" t="n">
         <v>5</v>
@@ -2337,12 +2337,12 @@
       </c>
       <c r="K1" s="9" t="inlineStr">
         <is>
-          <t>NEED /2000 cases (+5% loss)</t>
+          <t>NEED /2000 cases (lbs,+5% loss)</t>
         </is>
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>BUY QTY (MOQ-adj)</t>
+          <t>BUY QTY (MOQ-adj, buy unit)</t>
         </is>
       </c>
       <c r="M1" s="9" t="inlineStr">
@@ -2363,11 +2363,11 @@
         </is>
       </c>
       <c r="C2" s="10" t="n">
-        <v>96.8</v>
+        <v>807.8359</v>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E2" s="10" t="n">
@@ -2389,7 +2389,7 @@
       </c>
       <c r="J2" s="11" t="inlineStr"/>
       <c r="K2" s="10" t="n">
-        <v>1611.0268</v>
+        <v>13444.6816</v>
       </c>
       <c r="L2" s="10" t="n">
         <v>1612</v>
@@ -2410,11 +2410,11 @@
         </is>
       </c>
       <c r="C3" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.2504</v>
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E3" s="10" t="n">
@@ -2436,7 +2436,7 @@
       </c>
       <c r="J3" s="11" t="inlineStr"/>
       <c r="K3" s="10" t="n">
-        <v>1.89</v>
+        <v>4.1667</v>
       </c>
       <c r="L3" s="10" t="n">
         <v>55</v>
@@ -2457,11 +2457,11 @@
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.2504</v>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E4" s="10" t="n">
@@ -2483,7 +2483,7 @@
       </c>
       <c r="J4" s="11" t="inlineStr"/>
       <c r="K4" s="10" t="n">
-        <v>1.89</v>
+        <v>4.1667</v>
       </c>
       <c r="L4" s="10" t="n">
         <v>55</v>
@@ -2504,11 +2504,11 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>0.1908</v>
+        <v>0.4206</v>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E5" s="10" t="n">
@@ -2530,7 +2530,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr"/>
       <c r="K5" s="10" t="n">
-        <v>3.1752</v>
+        <v>7.0001</v>
       </c>
       <c r="L5" s="10" t="n">
         <v>25</v>
@@ -2551,11 +2551,11 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>0.0757</v>
+        <v>0.1669</v>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E6" s="10" t="n">
@@ -2577,7 +2577,7 @@
       </c>
       <c r="J6" s="11" t="inlineStr"/>
       <c r="K6" s="10" t="n">
-        <v>1.26</v>
+        <v>2.7778</v>
       </c>
       <c r="L6" s="10" t="n">
         <v>2</v>
@@ -2598,11 +2598,11 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.53</v>
+        <v>1.1684</v>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E7" s="10" t="n">
@@ -2624,7 +2624,7 @@
       </c>
       <c r="J7" s="11" t="inlineStr"/>
       <c r="K7" s="10" t="n">
-        <v>8.82</v>
+        <v>19.4448</v>
       </c>
       <c r="L7" s="10" t="n">
         <v>9</v>
@@ -2739,11 +2739,11 @@
         </is>
       </c>
       <c r="C10" s="10" t="n">
-        <v>0.32</v>
+        <v>2.6705</v>
       </c>
       <c r="D10" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E10" s="10" t="n">
@@ -2765,7 +2765,7 @@
       </c>
       <c r="J10" s="11" t="inlineStr"/>
       <c r="K10" s="10" t="n">
-        <v>5.3257</v>
+        <v>44.4452</v>
       </c>
       <c r="L10" s="10" t="n">
         <v>6</v>
@@ -2786,11 +2786,11 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.24</v>
+        <v>2.0029</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E11" s="10" t="n">
@@ -2812,7 +2812,7 @@
       </c>
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="10" t="n">
-        <v>3.9943</v>
+        <v>33.3339</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>4</v>
@@ -2833,11 +2833,11 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>0.038</v>
+        <v>0.3171</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
@@ -2859,7 +2859,7 @@
       </c>
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="10" t="n">
-        <v>0.6324</v>
+        <v>5.2779</v>
       </c>
       <c r="L12" s="10" t="n">
         <v>1</v>
@@ -2880,11 +2880,11 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>0.096</v>
+        <v>0.8012</v>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E13" s="10" t="n">
@@ -2906,7 +2906,7 @@
       </c>
       <c r="J13" s="11" t="inlineStr"/>
       <c r="K13" s="10" t="n">
-        <v>1.5977</v>
+        <v>13.3336</v>
       </c>
       <c r="L13" s="10" t="n">
         <v>2</v>
@@ -2927,11 +2927,11 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>0.192</v>
+        <v>1.6023</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E14" s="10" t="n">
@@ -2953,7 +2953,7 @@
       </c>
       <c r="J14" s="11" t="inlineStr"/>
       <c r="K14" s="10" t="n">
-        <v>3.1954</v>
+        <v>26.6671</v>
       </c>
       <c r="L14" s="10" t="n">
         <v>4</v>
@@ -3110,12 +3110,12 @@
       </c>
       <c r="K1" s="9" t="inlineStr">
         <is>
-          <t>NEED /2000 cases (+5% loss)</t>
+          <t>NEED /2000 cases (lbs,+5% loss)</t>
         </is>
       </c>
       <c r="L1" s="9" t="inlineStr">
         <is>
-          <t>BUY QTY (MOQ-adj)</t>
+          <t>BUY QTY (MOQ-adj, buy unit)</t>
         </is>
       </c>
       <c r="M1" s="9" t="inlineStr">
@@ -3136,11 +3136,11 @@
         </is>
       </c>
       <c r="C2" s="10" t="n">
-        <v>93.28</v>
+        <v>778.46</v>
       </c>
       <c r="D2" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E2" s="10" t="n">
@@ -3162,7 +3162,7 @@
       </c>
       <c r="J2" s="11" t="inlineStr"/>
       <c r="K2" s="10" t="n">
-        <v>1552.444</v>
+        <v>12955.7841</v>
       </c>
       <c r="L2" s="10" t="n">
         <v>1553</v>
@@ -3230,11 +3230,11 @@
         </is>
       </c>
       <c r="C4" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.2504</v>
       </c>
       <c r="D4" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E4" s="10" t="n">
@@ -3256,7 +3256,7 @@
       </c>
       <c r="J4" s="11" t="inlineStr"/>
       <c r="K4" s="10" t="n">
-        <v>1.89</v>
+        <v>4.1667</v>
       </c>
       <c r="L4" s="10" t="n">
         <v>55</v>
@@ -3277,11 +3277,11 @@
         </is>
       </c>
       <c r="C5" s="10" t="n">
-        <v>0.1136</v>
+        <v>0.2504</v>
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E5" s="10" t="n">
@@ -3303,7 +3303,7 @@
       </c>
       <c r="J5" s="11" t="inlineStr"/>
       <c r="K5" s="10" t="n">
-        <v>1.89</v>
+        <v>4.1667</v>
       </c>
       <c r="L5" s="10" t="n">
         <v>55</v>
@@ -3324,11 +3324,11 @@
         </is>
       </c>
       <c r="C6" s="10" t="n">
-        <v>0.3725</v>
+        <v>0.8212</v>
       </c>
       <c r="D6" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E6" s="10" t="n">
@@ -3350,7 +3350,7 @@
       </c>
       <c r="J6" s="11" t="inlineStr"/>
       <c r="K6" s="10" t="n">
-        <v>6.1992</v>
+        <v>13.6669</v>
       </c>
       <c r="L6" s="10" t="n">
         <v>25</v>
@@ -3371,11 +3371,11 @@
         </is>
       </c>
       <c r="C7" s="10" t="n">
-        <v>0.0757</v>
+        <v>0.1669</v>
       </c>
       <c r="D7" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E7" s="10" t="n">
@@ -3397,7 +3397,7 @@
       </c>
       <c r="J7" s="11" t="inlineStr"/>
       <c r="K7" s="10" t="n">
-        <v>1.26</v>
+        <v>2.7778</v>
       </c>
       <c r="L7" s="10" t="n">
         <v>2</v>
@@ -3418,11 +3418,11 @@
         </is>
       </c>
       <c r="C8" s="10" t="n">
-        <v>0.6814</v>
+        <v>1.5022</v>
       </c>
       <c r="D8" s="10" t="inlineStr">
         <is>
-          <t>kg</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E8" s="10" t="n">
@@ -3444,7 +3444,7 @@
       </c>
       <c r="J8" s="11" t="inlineStr"/>
       <c r="K8" s="10" t="n">
-        <v>11.34</v>
+        <v>25.0004</v>
       </c>
       <c r="L8" s="10" t="n">
         <v>12</v>
@@ -3559,11 +3559,11 @@
         </is>
       </c>
       <c r="C11" s="10" t="n">
-        <v>0.152</v>
+        <v>1.2685</v>
       </c>
       <c r="D11" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E11" s="10" t="n">
@@ -3585,7 +3585,7 @@
       </c>
       <c r="J11" s="11" t="inlineStr"/>
       <c r="K11" s="10" t="n">
-        <v>2.5297</v>
+        <v>21.1115</v>
       </c>
       <c r="L11" s="10" t="n">
         <v>3</v>
@@ -3606,11 +3606,11 @@
         </is>
       </c>
       <c r="C12" s="10" t="n">
-        <v>0.092</v>
+        <v>0.7678</v>
       </c>
       <c r="D12" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E12" s="10" t="n">
@@ -3632,7 +3632,7 @@
       </c>
       <c r="J12" s="11" t="inlineStr"/>
       <c r="K12" s="10" t="n">
-        <v>1.5311</v>
+        <v>12.778</v>
       </c>
       <c r="L12" s="10" t="n">
         <v>2</v>
@@ -3653,11 +3653,11 @@
         </is>
       </c>
       <c r="C13" s="10" t="n">
-        <v>0.112</v>
+        <v>0.9347</v>
       </c>
       <c r="D13" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E13" s="10" t="n">
@@ -3679,7 +3679,7 @@
       </c>
       <c r="J13" s="11" t="inlineStr"/>
       <c r="K13" s="10" t="n">
-        <v>1.864</v>
+        <v>15.5558</v>
       </c>
       <c r="L13" s="10" t="n">
         <v>2</v>
@@ -3700,11 +3700,11 @@
         </is>
       </c>
       <c r="C14" s="10" t="n">
-        <v>0.14</v>
+        <v>1.1684</v>
       </c>
       <c r="D14" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E14" s="10" t="n">
@@ -3726,7 +3726,7 @@
       </c>
       <c r="J14" s="11" t="inlineStr"/>
       <c r="K14" s="10" t="n">
-        <v>2.33</v>
+        <v>19.4448</v>
       </c>
       <c r="L14" s="10" t="n">
         <v>3</v>
@@ -3747,11 +3747,11 @@
         </is>
       </c>
       <c r="C15" s="10" t="n">
-        <v>0.152</v>
+        <v>1.2685</v>
       </c>
       <c r="D15" s="10" t="inlineStr">
         <is>
-          <t>gal</t>
+          <t>lbs</t>
         </is>
       </c>
       <c r="E15" s="10" t="n">
@@ -3773,7 +3773,7 @@
       </c>
       <c r="J15" s="11" t="inlineStr"/>
       <c r="K15" s="10" t="n">
-        <v>2.5297</v>
+        <v>21.1115</v>
       </c>
       <c r="L15" s="10" t="n">
         <v>3</v>
@@ -4223,7 +4223,7 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>- Base batch = 100 gal finished. RECIPE AMT is per 100 gal, expressed in each ingredient BUY UNIT so RECIPE UNIT = BUY UNIT (no g-&gt;kg conversion to get wrong).</t>
+          <t>- Base batch = 100 gal finished. RECIPE AMT is per 100 gal, in LBS for every ingredient. BUY UNIT kept per-ingredient (gal/lbs/kg); SG converts lbs-&gt;gal for the volume-bought liquids (water, flavors, chamomile).</t>
         </is>
       </c>
     </row>

</xml_diff>